<commit_message>
#167 Bottom Board Client BOM PT100 added
</commit_message>
<xml_diff>
--- a/Design-Files/LSS_Bottom_Board_v3.4/BOM/Client_BOM-LSS_Bottom_Board_v3.4.xlsx
+++ b/Design-Files/LSS_Bottom_Board_v3.4/BOM/Client_BOM-LSS_Bottom_Board_v3.4.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\ColeBenson-SmartMotors\Design-Files\LSS_Bottom_Board_v3.4\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ColeBenson-SmartMotors\Design-Files\LSS_Bottom_Board_v3.4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="197">
   <si>
     <t>#</t>
   </si>
@@ -633,6 +633,15 @@
       </rPr>
       <t># Symbol is used for these Resistors in PCB</t>
     </r>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>PT100</t>
+  </si>
+  <si>
+    <t>RTD Temp Sensor</t>
   </si>
 </sst>
 </file>
@@ -1300,7 +1309,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="7" customWidth="1"/>
@@ -1396,7 +1405,7 @@
     <row r="4" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="23">
-        <f t="shared" ref="B4:B39" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B40" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="25" t="s">
@@ -2553,31 +2562,61 @@
       </c>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
-      <c r="B40" s="10"/>
-      <c r="C40" s="21"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="14"/>
-      <c r="J40" s="14"/>
-      <c r="K40" s="19"/>
-    </row>
-    <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="23">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="C40" s="25" t="s">
+        <v>194</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="E40" s="18" t="s">
+        <v>196</v>
+      </c>
+      <c r="F40" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="G40" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="H40" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="I40" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="J40" s="17"/>
+      <c r="K40" s="17"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="6"/>
-      <c r="C41" s="22"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
-      <c r="J41" s="4"/>
-      <c r="K41" s="20"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="12"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="14"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="14"/>
+      <c r="J41" s="14"/>
+      <c r="K41" s="19"/>
+    </row>
+    <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1"/>
+      <c r="B42" s="6"/>
+      <c r="C42" s="22"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>